<commit_message>
Sync Mad Lib builder and Kahoot import to live lecture answers
Match the five Oct 14 Kahoot questions (hospital-themed options) so the
speaker builder picks the same winners the room just voted.
</commit_message>
<xml_diff>
--- a/kahoot-madlib.xlsx
+++ b/kahoot-madlib.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -666,37 +666,39 @@
       <c r="I8" s="19" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1" s="30">
-      <c r="A9" s="20" t="n">
-        <v>1</v>
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Mad Lib 1 of 5: Build ___. What kind of app?</t>
+        </is>
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>Mad Lib 1 of 5: Build ___. What kind of app?</t>
+          <t>A survival game where the boss is the night-float pager</t>
         </is>
       </c>
       <c r="C9" s="22" t="inlineStr">
         <is>
-          <t>An arcade game</t>
+          <t>A 'who's the real attending' imposter game</t>
         </is>
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>A trivia quiz</t>
+          <t>A fighting game where the final boss is an EHR downtime screen</t>
         </is>
       </c>
       <c r="E9" s="22" t="inlineStr">
         <is>
-          <t>A random generator</t>
-        </is>
-      </c>
-      <c r="F9" s="22" t="inlineStr">
-        <is>
-          <t>A tracker with charts</t>
-        </is>
-      </c>
-      <c r="G9" s="22" t="n">
+          <t>An intergalactic space medicine game</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="n">
         <v>20</v>
       </c>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>1,2,3,4</t>
+        </is>
+      </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
           <t>1,2,3,4</t>
@@ -705,37 +707,39 @@
       <c r="I9" s="1" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1" s="30">
-      <c r="A10" s="20" t="n">
-        <v>2</v>
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Mad Lib 2 of 5: It is for ___. Who uses it?</t>
+        </is>
       </c>
       <c r="B10" s="22" t="inlineStr">
         <is>
-          <t>Mad Lib 2 of 5: It is for ___. Who uses it?</t>
+          <t>Sleep-deprived interns who were just paged for a potassium of 3.3</t>
         </is>
       </c>
       <c r="C10" s="22" t="inlineStr">
         <is>
-          <t>Sleep-deprived interns</t>
+          <t>Night float residents who have not seen sunlight for days</t>
         </is>
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>Night float residents</t>
+          <t>Chief residents who are somehow still smiling</t>
         </is>
       </c>
       <c r="E10" s="22" t="inlineStr">
         <is>
-          <t>Chief residents</t>
-        </is>
-      </c>
-      <c r="F10" s="22" t="inlineStr">
-        <is>
-          <t>Attendings on rounds</t>
-        </is>
-      </c>
-      <c r="G10" s="22" t="n">
+          <t>Attendings who say 'I'll be quick' and then are not</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="n">
         <v>20</v>
       </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>1,2,3,4</t>
+        </is>
+      </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
           <t>1,2,3,4</t>
@@ -744,37 +748,39 @@
       <c r="I10" s="1" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1" s="30">
-      <c r="A11" s="20" t="n">
-        <v>3</v>
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Mad Lib 3 of 5: It ___. What does it do?</t>
+        </is>
       </c>
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>Mad Lib 3 of 5: It ___. What does it do?</t>
+          <t>Matches you with the consult service you most want to avoid</t>
         </is>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
-          <t>Predicts how your shift will go</t>
+          <t>Collects coffee, snacks, and rare moments of quiet, scored on survival</t>
         </is>
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Rates your coffee order</t>
+          <t>Assigns the right level of drama to each page, graded on calibration</t>
         </is>
       </c>
       <c r="E11" s="22" t="inlineStr">
         <is>
-          <t>Picks where the team eats lunch</t>
-        </is>
-      </c>
-      <c r="F11" s="22" t="inlineStr">
-        <is>
           <t>Assigns you a medical spirit animal</t>
         </is>
       </c>
-      <c r="G11" s="22" t="n">
+      <c r="F11" s="22" t="n">
         <v>20</v>
       </c>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>1,2,3,4</t>
+        </is>
+      </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
           <t>1,2,3,4</t>
@@ -783,37 +789,39 @@
       <c r="I11" s="1" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1" s="30">
-      <c r="A12" s="20" t="n">
-        <v>4</v>
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Mad Lib 4 of 5: What should it look like?</t>
+        </is>
       </c>
       <c r="B12" s="22" t="inlineStr">
         <is>
-          <t>Mad Lib 4 of 5: What should it look like?</t>
+          <t>A fluorescent-lit call room that gets progressively messier</t>
         </is>
       </c>
       <c r="C12" s="22" t="inlineStr">
         <is>
-          <t>Retro 8-bit arcade</t>
+          <t>An over-the-top hospital drama set (think Grey's Anatomy)</t>
         </is>
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>Pirate ship</t>
+          <t>A pixel art version of the work room at 2 am</t>
         </is>
       </c>
       <c r="E12" s="22" t="inlineStr">
         <is>
-          <t>Space mission</t>
-        </is>
-      </c>
-      <c r="F12" s="22" t="inlineStr">
-        <is>
-          <t>Cozy cafe</t>
-        </is>
-      </c>
-      <c r="G12" s="22" t="n">
+          <t>A haunted hospital with ghosts and unfinished notes</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="n">
         <v>20</v>
       </c>
+      <c r="G12" s="22" t="inlineStr">
+        <is>
+          <t>1,2,3,4</t>
+        </is>
+      </c>
       <c r="H12" s="23" t="inlineStr">
         <is>
           <t>1,2,3,4</t>
@@ -822,36 +830,38 @@
       <c r="I12" s="1" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1" s="30">
-      <c r="A13" s="20" t="n">
-        <v>5</v>
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>Mad Lib 5 of 5: Pick one twist.</t>
+        </is>
       </c>
       <c r="B13" s="22" t="inlineStr">
         <is>
-          <t>Mad Lib 5 of 5: Pick one twist.</t>
+          <t>A "surprise rapid response" that interrupts whatever you are doing</t>
         </is>
       </c>
       <c r="C13" s="22" t="inlineStr">
         <is>
-          <t>Confetti when you win</t>
+          <t>The game occasionally interrupts itself with a fake or broken page</t>
         </is>
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>Countdown to end of shift</t>
+          <t>Your final score is delivered in the style of a night float sign out</t>
         </is>
       </c>
       <c r="E13" s="22" t="inlineStr">
         <is>
-          <t>A daily dad joke</t>
-        </is>
-      </c>
-      <c r="F13" s="22" t="inlineStr">
-        <is>
-          <t>A hidden easter egg</t>
-        </is>
-      </c>
-      <c r="G13" s="22" t="n">
+          <t>A "coffee level" bar that drains over time and must be refilled</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="n">
         <v>20</v>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>1,2,3,4</t>
+        </is>
       </c>
       <c r="H13" s="23" t="inlineStr">
         <is>

</xml_diff>